<commit_message>
운동프로그램 갱신 2026-08-18  0:25:47.38
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v18.xlsx
+++ b/운동프로그램_6일_v18.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{721FE110-B732-4B30-A8F5-2007FAAB75A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53363033-9B3C-4C33-90E4-D4B2CE1A2455}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{721FE110-B732-4B30-A8F5-2007FAAB75A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7C648B-7B8F-4FCB-9073-F0742336333C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17565" yWindow="1980" windowWidth="17670" windowHeight="18480" tabRatio="883" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1217" uniqueCount="673">
   <si>
     <t>시작 중량 설정 — 5년 공백 후 복귀</t>
   </si>
@@ -15427,10 +15427,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -16490,7 +16486,7 @@
       </c>
       <c r="H15" s="61">
         <f ca="1">SUM(D15:D16,D19)</f>
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1">
@@ -16580,7 +16576,7 @@
       </c>
       <c r="B19" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A19)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A19)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A19)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A19)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A19)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A19)</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C19" s="59">
         <f>MROUND(SUMIFS(간접계수맵!$F$7:$F$57,간접계수맵!$C$7:$C$57,$A19),0.5)</f>
@@ -16588,7 +16584,7 @@
       </c>
       <c r="D19" s="60">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E19" s="7" t="str">
         <f t="shared" si="1"/>
@@ -16730,12 +16726,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C25" s="66"/>
       <c r="D25" s="67">
         <f ca="1">SUM(D5:D24)</f>
-        <v>204.5</v>
+        <v>201.5</v>
       </c>
       <c r="E25" s="66"/>
       <c r="F25" s="66"/>
@@ -18990,7 +18986,7 @@
       </c>
       <c r="E7" s="20">
         <f>수_하체A!$E$23</f>
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F7" s="20" t="s">
         <v>75</v>
@@ -19088,7 +19084,7 @@
       <c r="D12" s="28"/>
       <c r="E12" s="27">
         <f>SUM(E5:E11)</f>
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -19304,7 +19300,7 @@
         <v>126</v>
       </c>
       <c r="D6" s="20">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E6" s="20">
         <v>4</v>
@@ -19333,7 +19329,7 @@
         <v>126</v>
       </c>
       <c r="D7" s="26">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E7" s="20">
         <v>3</v>
@@ -19390,8 +19386,8 @@
       <c r="C9" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>144</v>
+      <c r="D9" s="20">
+        <v>20</v>
       </c>
       <c r="E9" s="20">
         <v>3</v>
@@ -19449,7 +19445,7 @@
         <v>128</v>
       </c>
       <c r="D11" s="26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" s="20">
         <v>3</v>
@@ -20242,7 +20238,7 @@
         <v>63</v>
       </c>
       <c r="E21" s="20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F21" s="26" t="s">
         <v>145</v>
@@ -20288,7 +20284,7 @@
       </c>
       <c r="E23" s="27">
         <f>SUM(E15:E22)</f>
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-18  0:29:37.75
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v18.xlsx
+++ b/운동프로그램_6일_v18.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{721FE110-B732-4B30-A8F5-2007FAAB75A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7C648B-7B8F-4FCB-9073-F0742336333C}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{721FE110-B732-4B30-A8F5-2007FAAB75A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{227D4087-DFF4-45A5-AF6E-05FCBA819130}"/>
   <bookViews>
-    <workbookView xWindow="17565" yWindow="1980" windowWidth="17670" windowHeight="18480" tabRatio="883" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="883" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -15275,14 +15275,14 @@
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -15425,6 +15425,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16214,7 +16218,7 @@
       <c r="F5" s="58" t="s">
         <v>420</v>
       </c>
-      <c r="G5" s="86" t="s">
+      <c r="G5" s="88" t="s">
         <v>421</v>
       </c>
       <c r="H5" s="61">
@@ -16249,7 +16253,7 @@
       <c r="F6" s="58" t="s">
         <v>422</v>
       </c>
-      <c r="G6" s="86"/>
+      <c r="G6" s="88"/>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1">
       <c r="A7" s="58" t="s">
@@ -16274,7 +16278,7 @@
       <c r="F7" s="58" t="s">
         <v>423</v>
       </c>
-      <c r="G7" s="86" t="s">
+      <c r="G7" s="88" t="s">
         <v>424</v>
       </c>
       <c r="H7" s="61">
@@ -16305,7 +16309,7 @@
       <c r="F8" s="58" t="s">
         <v>425</v>
       </c>
-      <c r="G8" s="86"/>
+      <c r="G8" s="88"/>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1">
       <c r="A9" s="58" t="s">
@@ -16330,7 +16334,7 @@
       <c r="F9" s="58" t="s">
         <v>426</v>
       </c>
-      <c r="G9" s="86"/>
+      <c r="G9" s="88"/>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1">
       <c r="A10" s="58" t="s">
@@ -16355,7 +16359,7 @@
       <c r="F10" s="58" t="s">
         <v>427</v>
       </c>
-      <c r="G10" s="86"/>
+      <c r="G10" s="88"/>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1">
       <c r="A11" s="58" t="s">
@@ -16486,7 +16490,7 @@
       </c>
       <c r="H15" s="61">
         <f ca="1">SUM(D15:D16,D19)</f>
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1">
@@ -16537,12 +16541,12 @@
       <c r="F17" s="58" t="s">
         <v>434</v>
       </c>
-      <c r="G17" s="86" t="s">
+      <c r="G17" s="88" t="s">
         <v>215</v>
       </c>
       <c r="H17" s="61">
         <f ca="1">SUM(D17:D18)</f>
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
@@ -16551,7 +16555,7 @@
       </c>
       <c r="B18" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A18)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A18)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A18)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A18)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A18)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A18)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C18" s="59">
         <f ca="1">MROUND(SUMIFS(간접계수맵!$F$7:$F$57,간접계수맵!$C$7:$C$57,$A18),0.5)</f>
@@ -16559,7 +16563,7 @@
       </c>
       <c r="D18" s="60">
         <f t="shared" ca="1" si="0"/>
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="E18" s="7" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -16568,7 +16572,7 @@
       <c r="F18" s="58" t="s">
         <v>435</v>
       </c>
-      <c r="G18" s="86"/>
+      <c r="G18" s="88"/>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1">
       <c r="A19" s="58" t="s">
@@ -16576,7 +16580,7 @@
       </c>
       <c r="B19" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A19)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A19)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A19)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A19)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A19)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A19)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C19" s="59">
         <f>MROUND(SUMIFS(간접계수맵!$F$7:$F$57,간접계수맵!$C$7:$C$57,$A19),0.5)</f>
@@ -16584,7 +16588,7 @@
       </c>
       <c r="D19" s="60">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E19" s="7" t="str">
         <f t="shared" si="1"/>
@@ -16726,12 +16730,12 @@
       </c>
       <c r="B25" s="15">
         <f>SUM(B5:B24)</f>
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C25" s="66"/>
       <c r="D25" s="67">
         <f ca="1">SUM(D5:D24)</f>
-        <v>201.5</v>
+        <v>202.5</v>
       </c>
       <c r="E25" s="66"/>
       <c r="F25" s="66"/>
@@ -18986,7 +18990,7 @@
       </c>
       <c r="E7" s="20">
         <f>수_하체A!$E$23</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="20" t="s">
         <v>75</v>
@@ -19084,7 +19088,7 @@
       <c r="D12" s="28"/>
       <c r="E12" s="27">
         <f>SUM(E5:E11)</f>
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
@@ -20211,7 +20215,7 @@
         <v>63</v>
       </c>
       <c r="E20" s="20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" s="26" t="s">
         <v>233</v>
@@ -20238,7 +20242,7 @@
         <v>63</v>
       </c>
       <c r="E21" s="20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="26" t="s">
         <v>145</v>
@@ -20284,7 +20288,7 @@
       </c>
       <c r="E23" s="27">
         <f>SUM(E15:E22)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -21502,28 +21506,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="86" t="s">
         <v>348</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="87" t="s">
         <v>349</v>
       </c>
-      <c r="B4" s="88"/>
-      <c r="C4" s="88"/>
-      <c r="D4" s="88"/>
-      <c r="E4" s="88"/>
-      <c r="F4" s="88"/>
-      <c r="G4" s="88"/>
-      <c r="H4" s="88"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="87"/>
+      <c r="H4" s="87"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="A6" s="48" t="s">

</xml_diff>